<commit_message>
data: publish 2026-09-11 daily operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-11-上海公交运营分析.xlsx
+++ b/data/export/2026-09-11-上海公交运营分析.xlsx
@@ -561,7 +561,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -710,7 +710,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>金杨路枣庄路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>川环南路妙境路</t>
+          <t>新川路川沙路</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>金杨路金桥路</t>
+          <t>平度路长岛路</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川环南路妙境路</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路枣庄路</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>新川路川沙路</t>
+          <t>新川路华城路</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>平度路长岛路</t>
+          <t>荷泽路长岛路</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路金桥路</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>金杨路金业路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川环南路妙境路</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>新川路妙境路</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>平度路长岛路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>川沙路南桥路</t>
+          <t>新川路华城路</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>金杨路枣庄路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川环南路妙境路</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>金杨路金桥路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>新川路川沙路</t>
+          <t>新川路妙境路</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>川环南路妙境路</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路枣庄路</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>新川路川沙路</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路枣庄路</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>新川路华城路</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr"/>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="M33" s="1" t="inlineStr">
         <is>
-          <t>长岛路台儿庄路</t>
+          <t>博兴路东陆路</t>
         </is>
       </c>
       <c r="N33" s="1" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>金杨路金桥路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>金杨路枣庄路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr"/>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="M38" s="1" t="inlineStr">
         <is>
-          <t>川环南路妙境路</t>
+          <t>新川路妙境路</t>
         </is>
       </c>
       <c r="N38" s="1" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>川沙路南桥路</t>
+          <t>新川路川沙路</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>平度路长岛路</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr"/>
@@ -3800,7 +3800,7 @@
       </c>
       <c r="M42" s="1" t="inlineStr">
         <is>
-          <t>新德西路德川路</t>
+          <t>德川路华夏东路</t>
         </is>
       </c>
       <c r="N42" s="1" t="inlineStr">
@@ -3923,12 +3923,12 @@
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>运行异常待查</t>
+          <t>疑似区间车</t>
         </is>
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>同向实际位置连续推进至迎春路长柳路附近后停止；约11分钟后在锦绣路梅花路附近形成反向连续轨迹（7个采样点），空间衔接符合中途折返</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr"/>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr"/>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="M46" s="1" t="inlineStr">
         <is>
-          <t>迎春路长柳路</t>
+          <t>丁香路锦绣路</t>
         </is>
       </c>
       <c r="N46" s="1" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>锦绣路世纪大道</t>
+          <t>锦绣路梅花路</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="M48" s="1" t="inlineStr">
         <is>
-          <t>康弘路康丽路</t>
+          <t>康丽路康弘路</t>
         </is>
       </c>
       <c r="N48" s="1" t="inlineStr">
@@ -4357,12 +4357,12 @@
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>运行异常待查</t>
+          <t>疑似区间车</t>
         </is>
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>同向实际位置连续推进至锦绣路世纪大道附近后停止；约10分钟后在锦绣路花木路附近形成反向连续轨迹（8个采样点），空间衔接符合中途折返</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr"/>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="M50" s="1" t="inlineStr">
         <is>
-          <t>锦绣路花木路</t>
+          <t>锦绣路世纪大道</t>
         </is>
       </c>
       <c r="N50" s="1" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="M51" s="1" t="inlineStr">
         <is>
-          <t>康沈路梓康路</t>
+          <t>关岳路周园路</t>
         </is>
       </c>
       <c r="N51" s="1" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>东靖路东沟路</t>
+          <t>浦东大道东波路</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>东靖路莱阳路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>康弘路康汇路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康汇路康恩路</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>康恩路康丽路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="M63" s="1" t="inlineStr">
         <is>
-          <t>迎春路芳甸路</t>
+          <t>锦绣路花木路</t>
         </is>
       </c>
       <c r="N63" s="1" t="inlineStr">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>康汇路康恩路</t>
+          <t>康恩路康丽路</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>浦东大道东波路</t>
+          <t>莱阳路东陆路</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>东靖路东沟路</t>
+          <t>东葛路东靖路</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康弘路康汇路</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>康丽路康恩路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路张杨北路</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -6266,7 +6266,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="M76" s="1" t="inlineStr">
         <is>
-          <t>白桦路明月路</t>
+          <t>丁香路锦绣路</t>
         </is>
       </c>
       <c r="N76" s="1" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>东靖路莱阳路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>康恩路康丽路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>东靖路张杨北路</t>
+          <t>东葛路东靖路</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -6646,7 +6646,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>康丽路康弘路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6724,7 +6724,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>康弘路康丽路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路张杨北路</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>康弘路康丽路</t>
+          <t>康丽路康恩路</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>康弘路康佳路（康桥卫生中心）</t>
+          <t>关岳路周园路</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路清溪路</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>和龙路花山路</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>丁香路合欢路</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>和龙路花山路</t>
+          <t>和龙路清溪路</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>丁香路合欢路</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>丁香路合欢路</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -7816,7 +7816,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -8050,7 +8050,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>大同路和龙路</t>
+          <t>杨高北路花山路</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr"/>
@@ -8196,7 +8196,7 @@
       </c>
       <c r="M100" s="1" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N100" s="1" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -8352,7 +8352,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>丁香路长柳路</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -8508,7 +8508,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>芳甸路杨高中路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -8742,7 +8742,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>大同路清溪路</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>丁香路金松路</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>和龙路花山路</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr"/>
@@ -9044,7 +9044,7 @@
       </c>
       <c r="M111" s="1" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>丁香路民生路</t>
         </is>
       </c>
       <c r="N111" s="1" t="inlineStr">
@@ -9122,7 +9122,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -9200,7 +9200,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -9356,7 +9356,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -9434,7 +9434,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -9512,7 +9512,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="M118" s="1" t="inlineStr">
         <is>
-          <t>丁香路金松路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N118" s="1" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -9746,7 +9746,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>芳甸路杨高中路</t>
+          <t>云山路灵山路</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>丁香路金松路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -9902,7 +9902,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>和龙路清溪路</t>
+          <t>大同路石家街（市七医院）</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -10058,7 +10058,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>丁香路金松路</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -10136,7 +10136,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>大同路和龙路</t>
+          <t>大同路花山路</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -10368,7 +10368,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -10446,7 +10446,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>丁香路金松路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -10680,7 +10680,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>和龙路花山路</t>
+          <t>和龙路清溪路</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -10718,13 +10718,13 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -10873,7 +10873,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -10951,7 +10951,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路清溪路</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -11029,7 +11029,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>和龙路花山路</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>丁香路合欢路</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -11185,7 +11185,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>和龙路花山路</t>
+          <t>和龙路清溪路</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -11263,7 +11263,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>丁香路合欢路</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -11341,7 +11341,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -11419,7 +11419,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>丁香路合欢路</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -11497,7 +11497,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -11653,7 +11653,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -11809,7 +11809,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>大同路和龙路</t>
+          <t>杨高北路花山路</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -11859,7 +11859,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr"/>
@@ -11877,7 +11877,7 @@
       </c>
       <c r="M15" s="1" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N15" s="1" t="inlineStr">
@@ -11955,7 +11955,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>丁香路长柳路</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -12111,7 +12111,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -12189,7 +12189,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -12267,7 +12267,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>芳甸路杨高中路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -12345,7 +12345,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -12423,7 +12423,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>大同路清溪路</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>丁香路金松路</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -12657,7 +12657,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>和龙路花山路</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -12707,7 +12707,7 @@
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr"/>
@@ -12725,7 +12725,7 @@
       </c>
       <c r="M26" s="1" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>丁香路民生路</t>
         </is>
       </c>
       <c r="N26" s="1" t="inlineStr">
@@ -12803,7 +12803,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -12881,7 +12881,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>丁香路合欢路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -13271,7 +13271,7 @@
       </c>
       <c r="M33" s="1" t="inlineStr">
         <is>
-          <t>丁香路金松路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N33" s="1" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -13427,7 +13427,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>芳甸路杨高中路</t>
+          <t>云山路灵山路</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -13505,7 +13505,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>丁香路金松路</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -13583,7 +13583,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>和龙路清溪路</t>
+          <t>大同路石家街（市七医院）</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -13739,7 +13739,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>丁香路民生路</t>
+          <t>丁香路金松路</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -13817,7 +13817,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>港城路地铁站</t>
+          <t>和龙路草高支路</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -13895,7 +13895,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>大同路和龙路</t>
+          <t>大同路花山路</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -14049,7 +14049,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>锦带路迎春路（浦东新区办公中心）</t>
+          <t>杨高中路云山路</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -14127,7 +14127,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>和龙路草高支路</t>
+          <t>大同路和龙路</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -14283,7 +14283,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>丁香路金松路</t>
+          <t>芳甸路杨高中路</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -14361,7 +14361,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>和龙路花山路</t>
+          <t>和龙路清溪路</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -14521,12 +14521,12 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>运行异常待查</t>
+          <t>疑似区间车</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>同向实际位置连续推进至迎春路长柳路附近后停止；约11分钟后在锦绣路梅花路附近形成反向连续轨迹（7个采样点），空间衔接符合中途折返</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr"/>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr"/>
@@ -14690,7 +14690,7 @@
       </c>
       <c r="M4" s="1" t="inlineStr">
         <is>
-          <t>迎春路长柳路</t>
+          <t>丁香路锦绣路</t>
         </is>
       </c>
       <c r="N4" s="1" t="inlineStr">
@@ -14768,7 +14768,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>锦绣路世纪大道</t>
+          <t>锦绣路梅花路</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -14818,7 +14818,7 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr"/>
@@ -14836,7 +14836,7 @@
       </c>
       <c r="M6" s="1" t="inlineStr">
         <is>
-          <t>康弘路康丽路</t>
+          <t>康丽路康弘路</t>
         </is>
       </c>
       <c r="N6" s="1" t="inlineStr">
@@ -14955,12 +14955,12 @@
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>运行异常待查</t>
+          <t>疑似区间车</t>
         </is>
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>同向实际位置连续推进至锦绣路世纪大道附近后停止；约10分钟后在锦绣路花木路附近形成反向连续轨迹（8个采样点），空间衔接符合中途折返</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr"/>
@@ -14978,7 +14978,7 @@
       </c>
       <c r="M8" s="1" t="inlineStr">
         <is>
-          <t>锦绣路花木路</t>
+          <t>锦绣路世纪大道</t>
         </is>
       </c>
       <c r="N8" s="1" t="inlineStr">
@@ -15044,7 +15044,7 @@
       </c>
       <c r="M9" s="1" t="inlineStr">
         <is>
-          <t>康沈路梓康路</t>
+          <t>关岳路周园路</t>
         </is>
       </c>
       <c r="N9" s="1" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -15198,7 +15198,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -15276,7 +15276,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>东靖路东沟路</t>
+          <t>浦东大道东波路</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -15354,7 +15354,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -15548,7 +15548,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>东靖路莱阳路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -15626,7 +15626,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>康弘路康汇路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -15782,7 +15782,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康汇路康恩路</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -15860,7 +15860,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>康恩路康丽路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -15928,7 +15928,7 @@
       </c>
       <c r="M21" s="1" t="inlineStr">
         <is>
-          <t>迎春路芳甸路</t>
+          <t>锦绣路花木路</t>
         </is>
       </c>
       <c r="N21" s="1" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>康汇路康恩路</t>
+          <t>康恩路康丽路</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -16084,7 +16084,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>浦东大道东波路</t>
+          <t>莱阳路东陆路</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -16240,7 +16240,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>东靖路东沟路</t>
+          <t>东葛路东靖路</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -16318,7 +16318,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康弘路康汇路</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -16630,7 +16630,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>康丽路康恩路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -16786,7 +16786,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路张杨北路</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -16864,7 +16864,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>康恩路康浦路</t>
+          <t>康弘路康佳路（康桥卫生中心）</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -16932,7 +16932,7 @@
       </c>
       <c r="M34" s="1" t="inlineStr">
         <is>
-          <t>白桦路明月路</t>
+          <t>丁香路锦绣路</t>
         </is>
       </c>
       <c r="N34" s="1" t="inlineStr">
@@ -17010,7 +17010,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>东靖路莱阳路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>康恩路康丽路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -17166,7 +17166,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>东靖路张杨北路</t>
+          <t>东葛路东靖路</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -17244,7 +17244,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>康丽路康弘路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -17322,7 +17322,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>康弘路康丽路</t>
+          <t>关岳路康达路</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -17400,7 +17400,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路张杨北路</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -17556,7 +17556,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>东高路张杨北路</t>
+          <t>东靖路东沟路</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -17634,7 +17634,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>康弘路康丽路</t>
+          <t>康丽路康恩路</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -17712,7 +17712,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>康弘路康佳路（康桥卫生中心）</t>
+          <t>关岳路周园路</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -17750,7 +17750,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -17905,7 +17905,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>金杨路枣庄路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -17983,7 +17983,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>川环南路妙境路</t>
+          <t>新川路川沙路</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -18061,7 +18061,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>金杨路金桥路</t>
+          <t>平度路长岛路</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -18139,7 +18139,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川环南路妙境路</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -18217,7 +18217,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路枣庄路</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -18295,7 +18295,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>新川路川沙路</t>
+          <t>新川路华城路</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -18373,7 +18373,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>平度路长岛路</t>
+          <t>荷泽路长岛路</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -18529,7 +18529,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路金桥路</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -18607,7 +18607,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>金杨路金业路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -18685,7 +18685,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川环南路妙境路</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -18841,7 +18841,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -18919,7 +18919,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -18997,7 +18997,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>新川路妙境路</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -19075,7 +19075,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>平度路长岛路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -19309,7 +19309,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>川沙路南桥路</t>
+          <t>新川路华城路</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -19387,7 +19387,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>金杨路枣庄路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -19543,7 +19543,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川环南路妙境路</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -19621,7 +19621,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>金杨路金桥路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -19699,7 +19699,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>新川路川沙路</t>
+          <t>新川路妙境路</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -19777,7 +19777,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>川环南路妙境路</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -19855,7 +19855,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路枣庄路</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -19933,7 +19933,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>新川路川沙路</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -20011,7 +20011,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路枣庄路</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -20089,7 +20089,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -20245,7 +20245,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>新川路华城路</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -20295,7 +20295,7 @@
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr"/>
@@ -20313,7 +20313,7 @@
       </c>
       <c r="M33" s="1" t="inlineStr">
         <is>
-          <t>长岛路台儿庄路</t>
+          <t>博兴路东陆路</t>
         </is>
       </c>
       <c r="N33" s="1" t="inlineStr">
@@ -20391,7 +20391,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>川环南路川沙路</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -20469,7 +20469,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>川沙客运站</t>
+          <t>川沙路南桥路</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -20547,7 +20547,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>金杨路金桥路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -20625,7 +20625,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>金杨路枣庄路</t>
+          <t>长岛路台儿庄路</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -20675,7 +20675,7 @@
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr"/>
@@ -20693,7 +20693,7 @@
       </c>
       <c r="M38" s="1" t="inlineStr">
         <is>
-          <t>川环南路妙境路</t>
+          <t>新川路妙境路</t>
         </is>
       </c>
       <c r="N38" s="1" t="inlineStr">
@@ -20771,7 +20771,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>川沙路南桥路</t>
+          <t>新川路川沙路</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -20849,7 +20849,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>平度路长岛路</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -20927,7 +20927,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>金杨路金口路</t>
+          <t>金杨路金业路</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -20977,7 +20977,7 @@
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>反方向current/next属于站点到站预测，未形成可验证的实际折返轨迹；不判区间车</t>
+          <t>出现反方向到站预测，但未满足连续位置、时间及空间衔接三项折返证据；不判区间车</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr"/>
@@ -20995,7 +20995,7 @@
       </c>
       <c r="M42" s="1" t="inlineStr">
         <is>
-          <t>新德西路德川路</t>
+          <t>德川路华夏东路</t>
         </is>
       </c>
       <c r="N42" s="1" t="inlineStr">

</xml_diff>